<commit_message>
antes de subir al naas
</commit_message>
<xml_diff>
--- a/last_version/ID-Dish-Catalogue_v2.xlsx
+++ b/last_version/ID-Dish-Catalogue_v2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unizares-my.sharepoint.com/personal/819658_unizar_es/Documents/_UNIZAR/GILAB/BSH excel/Qwen (tiene los cambios despues mail tereca)/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\AppData\Roaming\MobaXterm\slash\RemoteFiles\6358986_11_17\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="8_{1BEED36B-B2B9-4C4C-8304-17EEA6668E02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE89E692-4CDF-4761-8398-B8C8892DFC82}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D72C7CB-39C8-436C-AB96-33C3A2684CFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>